<commit_message>
Docs: gig worker flow released — production smoke results, tracker and open items
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-31.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-31.xlsx
@@ -6810,7 +6810,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>Test site (test.gokesari.com) since 31 Oct 2026</t>
+    <t>Production (gokesari.com) and Test site since 31 Oct 2026</t>
   </si>
   <si>
     <t>Live on the Test site</t>
@@ -6819,10 +6819,7 @@
     <t>#306</t>
   </si>
   <si>
-    <t>Not yet — goes with staging → main release PR #302 (owner window)</t>
-  </si>
-  <si>
-    <t>Production release (owner approval); Production database → migrate 0121 first</t>
+    <t>#302 (merged 31 Oct 2026 11:43 UTC; post-deploy check passed)</t>
   </si>
   <si>
     <t>NEW (not in 29 Oct)</t>
@@ -6846,6 +6843,9 @@
     <t>Aadhaar OTP against the live provider (Test-site keys answer only saved examples); consent wording legal review</t>
   </si>
   <si>
+    <t>See remaining scope</t>
+  </si>
+  <si>
     <t>src/server/services/rider-kyc.ts; src/server/kyc/adapters/{mock,sandbox-co}.ts; /delivery-partner/kyc</t>
   </si>
   <si>
@@ -15606,7 +15606,7 @@
     <t>GW-01..GW-11</t>
   </si>
   <si>
-    <t>Not yet (in #302)</t>
+    <t>#302</t>
   </si>
   <si>
     <t>Migration 0121 (split: core) applied to the Test database 31 Oct 08:38 UTC.</t>
@@ -49791,16 +49791,16 @@
         <v>142</v>
       </c>
       <c r="O337" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P337" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P337" s="11" t="s">
+      <c r="Q337" s="11" t="s">
         <v>2263</v>
       </c>
-      <c r="Q337" s="11" t="s">
+      <c r="R337" s="11" t="s">
         <v>2264</v>
-      </c>
-      <c r="R337" s="11" t="s">
-        <v>2265</v>
       </c>
     </row>
     <row r="338" spans="1:18" x14ac:dyDescent="0.25">
@@ -49811,16 +49811,16 @@
         <v>2252</v>
       </c>
       <c r="C338" s="5" t="s">
-        <v>2266</v>
+        <v>2265</v>
       </c>
       <c r="D338" s="11" t="s">
         <v>2254</v>
       </c>
       <c r="E338" s="11" t="s">
+        <v>2266</v>
+      </c>
+      <c r="F338" s="11" t="s">
         <v>2267</v>
-      </c>
-      <c r="F338" s="11" t="s">
-        <v>2268</v>
       </c>
       <c r="G338" s="11" t="s">
         <v>142</v>
@@ -49844,16 +49844,16 @@
         <v>2261</v>
       </c>
       <c r="N338" s="11" t="s">
+        <v>2268</v>
+      </c>
+      <c r="O338" s="11" t="s">
         <v>2269</v>
       </c>
-      <c r="O338" s="11" t="s">
+      <c r="P338" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P338" s="11" t="s">
+      <c r="Q338" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q338" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R338" s="11" t="s">
         <v>2270</v>
@@ -49903,13 +49903,13 @@
         <v>142</v>
       </c>
       <c r="O339" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P339" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P339" s="11" t="s">
+      <c r="Q339" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q339" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R339" s="11" t="s">
         <v>2274</v>
@@ -49959,13 +49959,13 @@
         <v>142</v>
       </c>
       <c r="O340" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P340" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P340" s="11" t="s">
+      <c r="Q340" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q340" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R340" s="11" t="s">
         <v>2278</v>
@@ -50015,13 +50015,13 @@
         <v>2283</v>
       </c>
       <c r="O341" s="11" t="s">
+        <v>2269</v>
+      </c>
+      <c r="P341" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P341" s="11" t="s">
+      <c r="Q341" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q341" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R341" s="11" t="s">
         <v>2284</v>
@@ -50071,13 +50071,13 @@
         <v>2288</v>
       </c>
       <c r="O342" s="11" t="s">
+        <v>2269</v>
+      </c>
+      <c r="P342" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P342" s="11" t="s">
+      <c r="Q342" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q342" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R342" s="11" t="s">
         <v>2289</v>
@@ -50127,13 +50127,13 @@
         <v>142</v>
       </c>
       <c r="O343" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P343" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P343" s="11" t="s">
+      <c r="Q343" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q343" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R343" s="11" t="s">
         <v>2293</v>
@@ -50183,13 +50183,13 @@
         <v>142</v>
       </c>
       <c r="O344" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P344" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P344" s="11" t="s">
+      <c r="Q344" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q344" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R344" s="11" t="s">
         <v>2297</v>
@@ -50239,13 +50239,13 @@
         <v>142</v>
       </c>
       <c r="O345" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P345" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P345" s="11" t="s">
+      <c r="Q345" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q345" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R345" s="11" t="s">
         <v>2301</v>
@@ -50295,13 +50295,13 @@
         <v>142</v>
       </c>
       <c r="O346" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P346" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P346" s="11" t="s">
+      <c r="Q346" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q346" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R346" s="11" t="s">
         <v>2305</v>
@@ -50351,13 +50351,13 @@
         <v>2309</v>
       </c>
       <c r="O347" s="11" t="s">
+        <v>2269</v>
+      </c>
+      <c r="P347" s="11" t="s">
         <v>2262</v>
       </c>
-      <c r="P347" s="11" t="s">
+      <c r="Q347" s="11" t="s">
         <v>2263</v>
-      </c>
-      <c r="Q347" s="11" t="s">
-        <v>2264</v>
       </c>
       <c r="R347" s="11" t="s">
         <v>2310</v>
@@ -69182,7 +69182,7 @@
         <v>5189</v>
       </c>
       <c r="J289" s="11" t="s">
-        <v>142</v>
+        <v>5189</v>
       </c>
       <c r="K289" s="11" t="s">
         <v>5190</v>
@@ -69220,7 +69220,7 @@
         <v>5195</v>
       </c>
       <c r="J290" s="11" t="s">
-        <v>142</v>
+        <v>5195</v>
       </c>
       <c r="K290" s="11" t="s">
         <v>5190</v>

</xml_diff>